<commit_message>
Fix typo in spreadsheet
</commit_message>
<xml_diff>
--- a/docs/CS858-F26-papers-stripped.xlsx
+++ b/docs/CS858-F26-papers-stripped.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uofwaterloo.sharepoint.com/sites/tm-math-ssg-mlsec/Shared Documents/General/MLSec-tutorial/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/asimwaheed/Documents/AllWork/Bots/cs858-wiki/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="660" documentId="11_A6B81843C1AE8CB9D7F3088654DFBA397E707E1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5268A3D0-5EBE-4472-B911-E35DA6356959}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F676B01-4AA7-264A-A01E-1318C8A08329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33420" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="33420" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UpdatedList" sheetId="1" r:id="rId1"/>
@@ -344,9 +344,6 @@
     <t>A Watermark for Large Language Models</t>
   </si>
   <si>
-    <t>Media Forensics and Proactive Provanance</t>
-  </si>
-  <si>
     <t>Tree-Ring Watermarks: Fingerprints for Diffusion Images that are Invisible and Robust</t>
   </si>
   <si>
@@ -616,12 +613,15 @@
   <si>
     <t>Model Theft Resistance (+ on-device private inference)  - Hardware</t>
   </si>
+  <si>
+    <t>Media Forensics and Proactive Provenance</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="38">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -847,6 +847,12 @@
     <font>
       <sz val="12"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1131,7 +1137,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="237">
+  <cellXfs count="238">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1431,24 +1437,219 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="7" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="7" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1473,203 +1674,56 @@
     <xf numFmtId="0" fontId="34" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
@@ -1683,60 +1737,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1963,16 +1972,16 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AB51"/>
-  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" style="31"/>
-    <col min="2" max="2" width="100.42578125" style="67" customWidth="1"/>
-    <col min="3" max="3" width="52.140625" style="67" customWidth="1"/>
-    <col min="4" max="4" width="40.7109375" style="31" customWidth="1"/>
-    <col min="5" max="5" width="90.85546875" style="31" customWidth="1"/>
+    <col min="1" max="1" width="12.5" style="31"/>
+    <col min="2" max="2" width="100.5" style="67" customWidth="1"/>
+    <col min="3" max="3" width="52.1640625" style="67" customWidth="1"/>
+    <col min="4" max="4" width="40.6640625" style="31" customWidth="1"/>
+    <col min="5" max="5" width="90.83203125" style="31" customWidth="1"/>
     <col min="6" max="6" width="72" style="31" customWidth="1"/>
-    <col min="7" max="7" width="83.42578125" style="31" customWidth="1"/>
-    <col min="8" max="16384" width="12.42578125" style="31"/>
+    <col min="7" max="7" width="83.5" style="31" customWidth="1"/>
+    <col min="8" max="16384" width="12.5" style="31"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="15" customHeight="1">
@@ -1997,34 +2006,34 @@
       </c>
     </row>
     <row r="2" spans="1:28" s="79" customFormat="1" ht="15" customHeight="1">
-      <c r="A2" s="169" t="s">
+      <c r="A2" s="172" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="170"/>
-      <c r="C2" s="170"/>
-      <c r="D2" s="170"/>
-      <c r="E2" s="171"/>
+      <c r="B2" s="173"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="174"/>
       <c r="F2" s="59"/>
       <c r="G2" s="78"/>
     </row>
     <row r="3" spans="1:28" ht="15" customHeight="1">
-      <c r="A3" s="154">
+      <c r="A3" s="133">
         <v>1</v>
       </c>
-      <c r="B3" s="208" t="s">
+      <c r="B3" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="180" t="s">
+      <c r="C3" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="154" t="s">
+      <c r="D3" s="133" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="104" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="59"/>
-      <c r="G3" s="205" t="s">
+      <c r="G3" s="131" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="80"/>
@@ -2050,15 +2059,15 @@
       <c r="AB3" s="80"/>
     </row>
     <row r="4" spans="1:28" ht="15" customHeight="1">
-      <c r="A4" s="231"/>
-      <c r="B4" s="208"/>
-      <c r="C4" s="181"/>
-      <c r="D4" s="231"/>
+      <c r="A4" s="134"/>
+      <c r="B4" s="144"/>
+      <c r="C4" s="161"/>
+      <c r="D4" s="134"/>
       <c r="E4" s="105" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="59"/>
-      <c r="G4" s="232"/>
+      <c r="G4" s="132"/>
       <c r="H4" s="80"/>
       <c r="I4" s="80"/>
       <c r="J4" s="80"/>
@@ -2082,14 +2091,14 @@
       <c r="AB4" s="80"/>
     </row>
     <row r="5" spans="1:28" ht="15" customHeight="1">
-      <c r="A5" s="154">
+      <c r="A5" s="133">
         <v>2</v>
       </c>
-      <c r="B5" s="178" t="s">
+      <c r="B5" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="181"/>
-      <c r="D5" s="154" t="s">
+      <c r="C5" s="161"/>
+      <c r="D5" s="133" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="104" t="s">
@@ -2124,10 +2133,10 @@
       <c r="AB5" s="30"/>
     </row>
     <row r="6" spans="1:28" ht="15" customHeight="1">
-      <c r="A6" s="231"/>
-      <c r="B6" s="179"/>
-      <c r="C6" s="181"/>
-      <c r="D6" s="231"/>
+      <c r="A6" s="134"/>
+      <c r="B6" s="146"/>
+      <c r="C6" s="161"/>
+      <c r="D6" s="134"/>
       <c r="E6" s="105" t="s">
         <v>18</v>
       </c>
@@ -2158,14 +2167,14 @@
       <c r="AB6" s="30"/>
     </row>
     <row r="7" spans="1:28" ht="15" customHeight="1">
-      <c r="A7" s="154">
+      <c r="A7" s="133">
         <v>3</v>
       </c>
-      <c r="B7" s="178" t="s">
+      <c r="B7" s="145" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="181"/>
-      <c r="D7" s="154" t="s">
+      <c r="C7" s="161"/>
+      <c r="D7" s="133" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="104" t="s">
@@ -2196,10 +2205,10 @@
       <c r="AB7" s="30"/>
     </row>
     <row r="8" spans="1:28" ht="15" customHeight="1">
-      <c r="A8" s="231"/>
-      <c r="B8" s="179"/>
-      <c r="C8" s="181"/>
-      <c r="D8" s="231"/>
+      <c r="A8" s="134"/>
+      <c r="B8" s="146"/>
+      <c r="C8" s="161"/>
+      <c r="D8" s="134"/>
       <c r="E8" s="106" t="s">
         <v>23</v>
       </c>
@@ -2228,14 +2237,14 @@
       <c r="AB8" s="30"/>
     </row>
     <row r="9" spans="1:28" ht="15" customHeight="1">
-      <c r="A9" s="154">
+      <c r="A9" s="133">
         <v>4</v>
       </c>
-      <c r="B9" s="203" t="s">
+      <c r="B9" s="137" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="181"/>
-      <c r="D9" s="154" t="s">
+      <c r="C9" s="161"/>
+      <c r="D9" s="133" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="104" t="s">
@@ -2270,10 +2279,10 @@
       <c r="AB9" s="30"/>
     </row>
     <row r="10" spans="1:28" ht="15" customHeight="1">
-      <c r="A10" s="231"/>
-      <c r="B10" s="204"/>
-      <c r="C10" s="182"/>
-      <c r="D10" s="231"/>
+      <c r="A10" s="134"/>
+      <c r="B10" s="138"/>
+      <c r="C10" s="162"/>
+      <c r="D10" s="134"/>
       <c r="E10" s="106" t="s">
         <v>29</v>
       </c>
@@ -2304,16 +2313,16 @@
       <c r="AB10" s="30"/>
     </row>
     <row r="11" spans="1:28" ht="15" customHeight="1">
-      <c r="A11" s="145">
+      <c r="A11" s="135">
         <v>5</v>
       </c>
-      <c r="B11" s="201" t="s">
+      <c r="B11" s="139" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="189" t="s">
+      <c r="C11" s="154" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="149" t="s">
+      <c r="D11" s="143" t="s">
         <v>33</v>
       </c>
       <c r="E11" s="107" t="s">
@@ -2346,10 +2355,10 @@
       <c r="AB11" s="30"/>
     </row>
     <row r="12" spans="1:28" ht="15" customHeight="1">
-      <c r="A12" s="233"/>
-      <c r="B12" s="202"/>
-      <c r="C12" s="190"/>
-      <c r="D12" s="233"/>
+      <c r="A12" s="136"/>
+      <c r="B12" s="140"/>
+      <c r="C12" s="155"/>
+      <c r="D12" s="136"/>
       <c r="E12" s="108" t="s">
         <v>36</v>
       </c>
@@ -2380,14 +2389,14 @@
       <c r="AB12" s="30"/>
     </row>
     <row r="13" spans="1:28" ht="15" customHeight="1">
-      <c r="A13" s="145">
+      <c r="A13" s="135">
         <v>6</v>
       </c>
-      <c r="B13" s="201" t="s">
+      <c r="B13" s="139" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="190"/>
-      <c r="D13" s="149" t="s">
+      <c r="C13" s="155"/>
+      <c r="D13" s="143" t="s">
         <v>39</v>
       </c>
       <c r="E13" s="109" t="s">
@@ -2420,10 +2429,10 @@
       <c r="AB13" s="30"/>
     </row>
     <row r="14" spans="1:28" ht="15" customHeight="1">
-      <c r="A14" s="233"/>
-      <c r="B14" s="202"/>
-      <c r="C14" s="190"/>
-      <c r="D14" s="233"/>
+      <c r="A14" s="136"/>
+      <c r="B14" s="140"/>
+      <c r="C14" s="155"/>
+      <c r="D14" s="136"/>
       <c r="E14" s="108" t="s">
         <v>42</v>
       </c>
@@ -2454,14 +2463,14 @@
       <c r="AB14" s="30"/>
     </row>
     <row r="15" spans="1:28" ht="15" customHeight="1">
-      <c r="A15" s="145">
+      <c r="A15" s="135">
         <v>7</v>
       </c>
-      <c r="B15" s="201" t="s">
+      <c r="B15" s="139" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="190"/>
-      <c r="D15" s="149" t="s">
+      <c r="C15" s="155"/>
+      <c r="D15" s="143" t="s">
         <v>45</v>
       </c>
       <c r="E15" s="110" t="s">
@@ -2494,10 +2503,10 @@
       <c r="AB15" s="30"/>
     </row>
     <row r="16" spans="1:28" ht="15" customHeight="1">
-      <c r="A16" s="233"/>
-      <c r="B16" s="202"/>
-      <c r="C16" s="190"/>
-      <c r="D16" s="233"/>
+      <c r="A16" s="136"/>
+      <c r="B16" s="140"/>
+      <c r="C16" s="155"/>
+      <c r="D16" s="136"/>
       <c r="E16" s="108" t="s">
         <v>48</v>
       </c>
@@ -2528,14 +2537,14 @@
       <c r="AB16" s="30"/>
     </row>
     <row r="17" spans="1:28" ht="15" customHeight="1">
-      <c r="A17" s="145">
+      <c r="A17" s="135">
         <v>8</v>
       </c>
-      <c r="B17" s="176" t="s">
+      <c r="B17" s="178" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="190"/>
-      <c r="D17" s="145" t="s">
+      <c r="C17" s="155"/>
+      <c r="D17" s="135" t="s">
         <v>51</v>
       </c>
       <c r="E17" s="110" t="s">
@@ -2567,10 +2576,10 @@
       <c r="AB17" s="30"/>
     </row>
     <row r="18" spans="1:28" ht="15" customHeight="1">
-      <c r="A18" s="233"/>
-      <c r="B18" s="177"/>
-      <c r="C18" s="191"/>
-      <c r="D18" s="233"/>
+      <c r="A18" s="136"/>
+      <c r="B18" s="179"/>
+      <c r="C18" s="156"/>
+      <c r="D18" s="136"/>
       <c r="E18" s="111" t="s">
         <v>54</v>
       </c>
@@ -2603,16 +2612,16 @@
       <c r="AB18" s="30"/>
     </row>
     <row r="19" spans="1:28" ht="15" customHeight="1">
-      <c r="A19" s="154">
+      <c r="A19" s="133">
         <v>9</v>
       </c>
-      <c r="B19" s="178" t="s">
+      <c r="B19" s="145" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="192" t="s">
+      <c r="C19" s="157" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="154" t="s">
+      <c r="D19" s="133" t="s">
         <v>58</v>
       </c>
       <c r="E19" s="104" t="s">
@@ -2645,10 +2654,10 @@
       <c r="AB19" s="30"/>
     </row>
     <row r="20" spans="1:28" ht="15" customHeight="1">
-      <c r="A20" s="231"/>
-      <c r="B20" s="179"/>
-      <c r="C20" s="193"/>
-      <c r="D20" s="231"/>
+      <c r="A20" s="134"/>
+      <c r="B20" s="146"/>
+      <c r="C20" s="158"/>
+      <c r="D20" s="134"/>
       <c r="E20" s="105" t="s">
         <v>61</v>
       </c>
@@ -2679,14 +2688,14 @@
       <c r="AB20" s="30"/>
     </row>
     <row r="21" spans="1:28" ht="15" customHeight="1">
-      <c r="A21" s="154">
+      <c r="A21" s="133">
         <v>10</v>
       </c>
-      <c r="B21" s="178" t="s">
+      <c r="B21" s="145" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="193"/>
-      <c r="D21" s="175" t="s">
+      <c r="C21" s="158"/>
+      <c r="D21" s="170" t="s">
         <v>64</v>
       </c>
       <c r="E21" s="104" t="s">
@@ -2719,10 +2728,10 @@
       <c r="AB21" s="30"/>
     </row>
     <row r="22" spans="1:28" ht="15" customHeight="1">
-      <c r="A22" s="231"/>
-      <c r="B22" s="179"/>
-      <c r="C22" s="194"/>
-      <c r="D22" s="231"/>
+      <c r="A22" s="134"/>
+      <c r="B22" s="146"/>
+      <c r="C22" s="159"/>
+      <c r="D22" s="134"/>
       <c r="E22" s="112" t="s">
         <v>67</v>
       </c>
@@ -2753,16 +2762,16 @@
       <c r="AB22" s="30"/>
     </row>
     <row r="23" spans="1:28" ht="15" customHeight="1">
-      <c r="A23" s="145">
+      <c r="A23" s="135">
         <v>11</v>
       </c>
-      <c r="B23" s="206" t="s">
+      <c r="B23" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="195" t="s">
+      <c r="C23" s="147" t="s">
         <v>70</v>
       </c>
-      <c r="D23" s="145" t="s">
+      <c r="D23" s="135" t="s">
         <v>71</v>
       </c>
       <c r="E23" s="110" t="s">
@@ -2796,10 +2805,10 @@
       <c r="AB23" s="80"/>
     </row>
     <row r="24" spans="1:28" ht="15" customHeight="1">
-      <c r="A24" s="233"/>
-      <c r="B24" s="207"/>
-      <c r="C24" s="196"/>
-      <c r="D24" s="233"/>
+      <c r="A24" s="136"/>
+      <c r="B24" s="142"/>
+      <c r="C24" s="148"/>
+      <c r="D24" s="136"/>
       <c r="E24" s="108" t="s">
         <v>75</v>
       </c>
@@ -2832,14 +2841,14 @@
       <c r="AB24" s="80"/>
     </row>
     <row r="25" spans="1:28" ht="15" customHeight="1">
-      <c r="A25" s="145">
+      <c r="A25" s="135">
         <v>12</v>
       </c>
-      <c r="B25" s="206" t="s">
+      <c r="B25" s="141" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="196"/>
-      <c r="D25" s="145" t="s">
+      <c r="C25" s="148"/>
+      <c r="D25" s="135" t="s">
         <v>79</v>
       </c>
       <c r="E25" s="110" t="s">
@@ -2869,10 +2878,10 @@
       <c r="AB25" s="30"/>
     </row>
     <row r="26" spans="1:28" ht="15" customHeight="1">
-      <c r="A26" s="233"/>
-      <c r="B26" s="207"/>
-      <c r="C26" s="197"/>
-      <c r="D26" s="233"/>
+      <c r="A26" s="136"/>
+      <c r="B26" s="142"/>
+      <c r="C26" s="149"/>
+      <c r="D26" s="136"/>
       <c r="E26" s="108" t="s">
         <v>81</v>
       </c>
@@ -2903,16 +2912,16 @@
       <c r="AB26" s="30"/>
     </row>
     <row r="27" spans="1:28" ht="15" customHeight="1">
-      <c r="A27" s="154">
+      <c r="A27" s="133">
         <v>13</v>
       </c>
-      <c r="B27" s="203" t="s">
+      <c r="B27" s="137" t="s">
         <v>83</v>
       </c>
-      <c r="C27" s="198" t="s">
+      <c r="C27" s="150" t="s">
         <v>84</v>
       </c>
-      <c r="D27" s="154" t="s">
+      <c r="D27" s="133" t="s">
         <v>85</v>
       </c>
       <c r="E27" s="104" t="s">
@@ -2949,10 +2958,10 @@
       <c r="AB27" s="30"/>
     </row>
     <row r="28" spans="1:28" ht="15" customHeight="1">
-      <c r="A28" s="231"/>
-      <c r="B28" s="204"/>
-      <c r="C28" s="199"/>
-      <c r="D28" s="155"/>
+      <c r="A28" s="134"/>
+      <c r="B28" s="138"/>
+      <c r="C28" s="151"/>
+      <c r="D28" s="153"/>
       <c r="E28" s="113" t="s">
         <v>90</v>
       </c>
@@ -2982,14 +2991,14 @@
       <c r="AB28" s="30"/>
     </row>
     <row r="29" spans="1:28" ht="15" customHeight="1">
-      <c r="A29" s="154">
+      <c r="A29" s="133">
         <v>14</v>
       </c>
-      <c r="B29" s="178" t="s">
+      <c r="B29" s="145" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="199"/>
-      <c r="D29" s="154" t="s">
+      <c r="C29" s="151"/>
+      <c r="D29" s="133" t="s">
         <v>93</v>
       </c>
       <c r="E29" s="104" t="s">
@@ -3020,10 +3029,10 @@
       <c r="AB29" s="30"/>
     </row>
     <row r="30" spans="1:28" ht="15" customHeight="1">
-      <c r="A30" s="231"/>
-      <c r="B30" s="179"/>
-      <c r="C30" s="199"/>
-      <c r="D30" s="155"/>
+      <c r="A30" s="134"/>
+      <c r="B30" s="146"/>
+      <c r="C30" s="151"/>
+      <c r="D30" s="153"/>
       <c r="E30" s="105" t="s">
         <v>95</v>
       </c>
@@ -3051,46 +3060,46 @@
       <c r="AB30" s="30"/>
     </row>
     <row r="31" spans="1:28" ht="15" customHeight="1">
-      <c r="A31" s="154">
+      <c r="A31" s="133">
         <v>15</v>
       </c>
-      <c r="B31" s="203" t="s">
+      <c r="B31" s="137" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="199"/>
-      <c r="D31" s="154" t="s">
+      <c r="C31" s="151"/>
+      <c r="D31" s="237" t="s">
+        <v>183</v>
+      </c>
+      <c r="E31" s="114" t="s">
         <v>97</v>
-      </c>
-      <c r="E31" s="114" t="s">
-        <v>98</v>
       </c>
       <c r="F31" s="63"/>
       <c r="G31" s="70"/>
     </row>
     <row r="32" spans="1:28" ht="15" customHeight="1">
-      <c r="A32" s="231"/>
-      <c r="B32" s="204"/>
-      <c r="C32" s="199"/>
-      <c r="D32" s="155"/>
+      <c r="A32" s="134"/>
+      <c r="B32" s="138"/>
+      <c r="C32" s="151"/>
+      <c r="D32" s="153"/>
       <c r="E32" s="115" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F32" s="59"/>
       <c r="G32" s="70"/>
     </row>
     <row r="33" spans="1:28" ht="15" customHeight="1">
-      <c r="A33" s="154">
+      <c r="A33" s="133">
         <v>16</v>
       </c>
-      <c r="B33" s="178" t="s">
+      <c r="B33" s="145" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="151"/>
+      <c r="D33" s="133" t="s">
         <v>100</v>
       </c>
-      <c r="C33" s="199"/>
-      <c r="D33" s="154" t="s">
+      <c r="E33" s="104" t="s">
         <v>101</v>
-      </c>
-      <c r="E33" s="104" t="s">
-        <v>102</v>
       </c>
       <c r="F33" s="59"/>
       <c r="H33" s="30"/>
@@ -3116,16 +3125,16 @@
       <c r="AB33" s="30"/>
     </row>
     <row r="34" spans="1:28" ht="15" customHeight="1">
-      <c r="A34" s="231"/>
-      <c r="B34" s="179"/>
-      <c r="C34" s="200"/>
-      <c r="D34" s="231"/>
+      <c r="A34" s="134"/>
+      <c r="B34" s="146"/>
+      <c r="C34" s="152"/>
+      <c r="D34" s="134"/>
       <c r="E34" s="113" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F34" s="64"/>
       <c r="G34" s="71" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H34" s="30"/>
       <c r="I34" s="30"/>
@@ -3150,13 +3159,13 @@
       <c r="AB34" s="30"/>
     </row>
     <row r="35" spans="1:28" ht="15" customHeight="1">
-      <c r="A35" s="172" t="s">
-        <v>105</v>
-      </c>
-      <c r="B35" s="173"/>
-      <c r="C35" s="173"/>
-      <c r="D35" s="173"/>
-      <c r="E35" s="174"/>
+      <c r="A35" s="175" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" s="176"/>
+      <c r="C35" s="176"/>
+      <c r="D35" s="176"/>
+      <c r="E35" s="177"/>
       <c r="F35" s="72"/>
       <c r="G35" s="73"/>
       <c r="H35" s="30"/>
@@ -3182,20 +3191,20 @@
       <c r="AB35" s="30"/>
     </row>
     <row r="36" spans="1:28" ht="15" customHeight="1">
-      <c r="A36" s="154">
+      <c r="A36" s="133">
         <v>17</v>
       </c>
-      <c r="B36" s="186" t="s">
+      <c r="B36" s="168" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" s="184" t="s">
         <v>106</v>
       </c>
-      <c r="C36" s="151" t="s">
+      <c r="D36" s="170" t="s">
         <v>107</v>
       </c>
-      <c r="D36" s="175" t="s">
+      <c r="E36" s="116" t="s">
         <v>108</v>
-      </c>
-      <c r="E36" s="116" t="s">
-        <v>109</v>
       </c>
       <c r="F36" s="74"/>
       <c r="G36" s="72" t="s">
@@ -3224,14 +3233,14 @@
       <c r="AB36" s="30"/>
     </row>
     <row r="37" spans="1:28" ht="15" customHeight="1">
-      <c r="A37" s="161"/>
-      <c r="B37" s="187"/>
-      <c r="C37" s="152"/>
-      <c r="D37" s="188"/>
+      <c r="A37" s="192"/>
+      <c r="B37" s="169"/>
+      <c r="C37" s="185"/>
+      <c r="D37" s="171"/>
       <c r="E37" s="117"/>
       <c r="F37" s="58"/>
       <c r="G37" s="75" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H37" s="30"/>
       <c r="I37" s="30"/>
@@ -3256,18 +3265,18 @@
       <c r="AB37" s="30"/>
     </row>
     <row r="38" spans="1:28" ht="15" customHeight="1">
-      <c r="A38" s="154">
+      <c r="A38" s="133">
         <v>18</v>
       </c>
-      <c r="B38" s="156" t="s">
+      <c r="B38" s="187" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" s="185"/>
+      <c r="D38" s="133" t="s">
         <v>111</v>
       </c>
-      <c r="C38" s="152"/>
-      <c r="D38" s="154" t="s">
+      <c r="E38" s="118" t="s">
         <v>112</v>
-      </c>
-      <c r="E38" s="118" t="s">
-        <v>113</v>
       </c>
       <c r="F38" s="58"/>
       <c r="G38" s="75"/>
@@ -3294,10 +3303,10 @@
       <c r="AB38" s="30"/>
     </row>
     <row r="39" spans="1:28" ht="15" customHeight="1">
-      <c r="A39" s="155"/>
-      <c r="B39" s="157"/>
-      <c r="C39" s="153"/>
-      <c r="D39" s="155"/>
+      <c r="A39" s="153"/>
+      <c r="B39" s="188"/>
+      <c r="C39" s="186"/>
+      <c r="D39" s="153"/>
       <c r="E39" s="119"/>
       <c r="F39" s="75"/>
       <c r="G39" s="76"/>
@@ -3324,24 +3333,24 @@
       <c r="AB39" s="30"/>
     </row>
     <row r="40" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A40" s="135">
+      <c r="A40" s="163">
         <v>19</v>
       </c>
-      <c r="B40" s="184" t="s">
+      <c r="B40" s="165" t="s">
+        <v>113</v>
+      </c>
+      <c r="C40" s="206" t="s">
         <v>114</v>
       </c>
-      <c r="C40" s="139" t="s">
+      <c r="D40" s="163" t="s">
+        <v>107</v>
+      </c>
+      <c r="E40" s="120" t="s">
         <v>115</v>
-      </c>
-      <c r="D40" s="135" t="s">
-        <v>108</v>
-      </c>
-      <c r="E40" s="120" t="s">
-        <v>116</v>
       </c>
       <c r="F40" s="85"/>
       <c r="G40" s="86" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H40" s="87"/>
       <c r="I40" s="87"/>
@@ -3366,16 +3375,16 @@
       <c r="AB40" s="87"/>
     </row>
     <row r="41" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A41" s="183"/>
-      <c r="B41" s="185"/>
-      <c r="C41" s="140"/>
-      <c r="D41" s="136"/>
+      <c r="A41" s="164"/>
+      <c r="B41" s="166"/>
+      <c r="C41" s="207"/>
+      <c r="D41" s="167"/>
       <c r="E41" s="121" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F41" s="85"/>
       <c r="G41" s="89" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H41" s="87"/>
       <c r="I41" s="87"/>
@@ -3400,18 +3409,18 @@
       <c r="AB41" s="87"/>
     </row>
     <row r="42" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A42" s="135">
+      <c r="A42" s="163">
         <v>20</v>
       </c>
-      <c r="B42" s="166" t="s">
+      <c r="B42" s="197" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" s="207"/>
+      <c r="D42" s="163" t="s">
+        <v>111</v>
+      </c>
+      <c r="E42" s="122" t="s">
         <v>119</v>
-      </c>
-      <c r="C42" s="140"/>
-      <c r="D42" s="135" t="s">
-        <v>112</v>
-      </c>
-      <c r="E42" s="122" t="s">
-        <v>120</v>
       </c>
       <c r="F42" s="85"/>
       <c r="G42" s="89"/>
@@ -3438,10 +3447,10 @@
       <c r="AB42" s="87"/>
     </row>
     <row r="43" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A43" s="136"/>
-      <c r="B43" s="167"/>
-      <c r="C43" s="141"/>
-      <c r="D43" s="136"/>
+      <c r="A43" s="167"/>
+      <c r="B43" s="198"/>
+      <c r="C43" s="208"/>
+      <c r="D43" s="167"/>
       <c r="E43" s="123"/>
       <c r="F43" s="90"/>
       <c r="G43" s="91"/>
@@ -3468,20 +3477,20 @@
       <c r="AB43" s="87"/>
     </row>
     <row r="44" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A44" s="133">
+      <c r="A44" s="199">
         <v>21</v>
       </c>
-      <c r="B44" s="137" t="s">
+      <c r="B44" s="204" t="s">
+        <v>120</v>
+      </c>
+      <c r="C44" s="209" t="s">
         <v>121</v>
       </c>
-      <c r="C44" s="142" t="s">
+      <c r="D44" s="199" t="s">
+        <v>107</v>
+      </c>
+      <c r="E44" s="124" t="s">
         <v>122</v>
-      </c>
-      <c r="D44" s="133" t="s">
-        <v>108</v>
-      </c>
-      <c r="E44" s="124" t="s">
-        <v>123</v>
       </c>
       <c r="F44" s="92"/>
       <c r="G44" s="93"/>
@@ -3508,14 +3517,14 @@
       <c r="AB44" s="94"/>
     </row>
     <row r="45" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A45" s="168"/>
-      <c r="B45" s="138"/>
-      <c r="C45" s="143"/>
-      <c r="D45" s="134"/>
+      <c r="A45" s="200"/>
+      <c r="B45" s="205"/>
+      <c r="C45" s="210"/>
+      <c r="D45" s="201"/>
       <c r="E45" s="125"/>
       <c r="F45" s="96"/>
       <c r="G45" s="97" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H45" s="94"/>
       <c r="I45" s="94"/>
@@ -3540,22 +3549,22 @@
       <c r="AB45" s="94"/>
     </row>
     <row r="46" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A46" s="133">
+      <c r="A46" s="199">
         <v>22</v>
       </c>
-      <c r="B46" s="131" t="s">
+      <c r="B46" s="202" t="s">
+        <v>124</v>
+      </c>
+      <c r="C46" s="210"/>
+      <c r="D46" s="199" t="s">
+        <v>111</v>
+      </c>
+      <c r="E46" s="126" t="s">
         <v>125</v>
-      </c>
-      <c r="C46" s="143"/>
-      <c r="D46" s="133" t="s">
-        <v>112</v>
-      </c>
-      <c r="E46" s="126" t="s">
-        <v>126</v>
       </c>
       <c r="F46" s="98"/>
       <c r="G46" s="92" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H46" s="94"/>
       <c r="I46" s="94"/>
@@ -3580,32 +3589,32 @@
       <c r="AB46" s="94"/>
     </row>
     <row r="47" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A47" s="134"/>
-      <c r="B47" s="132"/>
-      <c r="C47" s="144"/>
-      <c r="D47" s="134"/>
+      <c r="A47" s="201"/>
+      <c r="B47" s="203"/>
+      <c r="C47" s="211"/>
+      <c r="D47" s="201"/>
       <c r="E47" s="127"/>
       <c r="F47" s="99"/>
     </row>
     <row r="48" spans="1:28" ht="15" customHeight="1">
-      <c r="A48" s="145">
+      <c r="A48" s="135">
         <v>23</v>
       </c>
-      <c r="B48" s="164" t="s">
+      <c r="B48" s="195" t="s">
+        <v>127</v>
+      </c>
+      <c r="C48" s="189" t="s">
         <v>128</v>
       </c>
-      <c r="C48" s="158" t="s">
+      <c r="D48" s="143" t="s">
+        <v>107</v>
+      </c>
+      <c r="E48" s="128" t="s">
         <v>129</v>
-      </c>
-      <c r="D48" s="149" t="s">
-        <v>108</v>
-      </c>
-      <c r="E48" s="128" t="s">
-        <v>130</v>
       </c>
       <c r="F48" s="57"/>
       <c r="G48" s="75" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H48" s="30"/>
       <c r="I48" s="30"/>
@@ -3630,16 +3639,16 @@
       <c r="AB48" s="30"/>
     </row>
     <row r="49" spans="1:28" ht="15" customHeight="1">
-      <c r="A49" s="163"/>
-      <c r="B49" s="165"/>
-      <c r="C49" s="159"/>
-      <c r="D49" s="162"/>
+      <c r="A49" s="194"/>
+      <c r="B49" s="196"/>
+      <c r="C49" s="190"/>
+      <c r="D49" s="193"/>
       <c r="E49" s="129" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F49" s="69"/>
       <c r="G49" s="75" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H49" s="30"/>
       <c r="I49" s="30"/>
@@ -3664,25 +3673,25 @@
       <c r="AB49" s="30"/>
     </row>
     <row r="50" spans="1:28" ht="15" customHeight="1">
-      <c r="A50" s="145">
+      <c r="A50" s="135">
         <v>24</v>
       </c>
-      <c r="B50" s="147" t="s">
+      <c r="B50" s="181" t="s">
+        <v>133</v>
+      </c>
+      <c r="C50" s="190"/>
+      <c r="D50" s="143" t="s">
+        <v>111</v>
+      </c>
+      <c r="E50" s="130" t="s">
         <v>134</v>
-      </c>
-      <c r="C50" s="159"/>
-      <c r="D50" s="149" t="s">
-        <v>112</v>
-      </c>
-      <c r="E50" s="130" t="s">
-        <v>135</v>
       </c>
       <c r="F50" s="77"/>
       <c r="G50" s="72" t="s">
+        <v>135</v>
+      </c>
+      <c r="H50" s="75" t="s">
         <v>136</v>
-      </c>
-      <c r="H50" s="75" t="s">
-        <v>137</v>
       </c>
       <c r="I50" s="30"/>
       <c r="J50" s="30"/>
@@ -3706,16 +3715,16 @@
       <c r="AB50" s="30"/>
     </row>
     <row r="51" spans="1:28" ht="15" customHeight="1">
-      <c r="A51" s="146"/>
-      <c r="B51" s="148"/>
-      <c r="C51" s="160"/>
-      <c r="D51" s="150"/>
+      <c r="A51" s="180"/>
+      <c r="B51" s="182"/>
+      <c r="C51" s="191"/>
+      <c r="D51" s="183"/>
       <c r="E51" s="129" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F51" s="69"/>
       <c r="G51" s="69" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H51" s="30"/>
       <c r="I51" s="30"/>
@@ -3741,6 +3750,74 @@
     </row>
   </sheetData>
   <mergeCells count="84">
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C40:C43"/>
+    <mergeCell ref="C44:C47"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C36:C39"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C48:C51"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="A42:A43"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="C3:C10"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C11:C18"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C23:C26"/>
+    <mergeCell ref="C27:C34"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B33:B34"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="A13:A14"/>
@@ -3757,74 +3834,6 @@
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="C23:C26"/>
-    <mergeCell ref="C27:C34"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="C11:C18"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="C3:C10"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C36:C39"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C48:C51"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="A48:A49"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="A42:A43"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="A44:A45"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C40:C43"/>
-    <mergeCell ref="C44:C47"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -3942,14 +3951,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" customWidth="1"/>
-    <col min="2" max="2" width="85.28515625" customWidth="1"/>
-    <col min="3" max="3" width="47.7109375" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="2" max="2" width="85.33203125" customWidth="1"/>
+    <col min="3" max="3" width="47.6640625" customWidth="1"/>
     <col min="4" max="4" width="87" customWidth="1"/>
-    <col min="5" max="5" width="95.7109375" customWidth="1"/>
-    <col min="6" max="26" width="8.85546875" customWidth="1"/>
+    <col min="5" max="5" width="95.6640625" customWidth="1"/>
+    <col min="6" max="26" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -3980,7 +3989,7 @@
       <c r="Y1" s="4"/>
       <c r="Z1" s="4"/>
     </row>
-    <row r="2" spans="1:26" ht="15.95">
+    <row r="2" spans="1:26" ht="16">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -3988,10 +3997,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>141</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>5</v>
@@ -4018,7 +4027,7 @@
       <c r="Y2" s="8"/>
       <c r="Z2" s="8"/>
     </row>
-    <row r="3" spans="1:26" ht="15.95">
+    <row r="3" spans="1:26" ht="16">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -4026,10 +4035,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="33" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="34" t="s">
         <v>142</v>
-      </c>
-      <c r="D3" s="34" t="s">
-        <v>143</v>
       </c>
       <c r="E3" s="35" t="s">
         <v>10</v>
@@ -4057,21 +4066,21 @@
       <c r="Z3" s="10"/>
     </row>
     <row r="4" spans="1:26">
-      <c r="A4" s="218">
+      <c r="A4" s="212">
         <f>SUM(A3+1)</f>
         <v>2</v>
       </c>
-      <c r="B4" s="226" t="s">
+      <c r="B4" s="214" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="227" t="s">
+      <c r="C4" s="216" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="E4" s="218" t="s">
         <v>145</v>
-      </c>
-      <c r="E4" s="219" t="s">
-        <v>146</v>
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
@@ -4096,13 +4105,13 @@
       <c r="Z4" s="11"/>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A5" s="234"/>
-      <c r="B5" s="235"/>
-      <c r="C5" s="236"/>
+      <c r="A5" s="213"/>
+      <c r="B5" s="215"/>
+      <c r="C5" s="217"/>
       <c r="D5" s="36" t="s">
-        <v>147</v>
-      </c>
-      <c r="E5" s="234"/>
+        <v>146</v>
+      </c>
+      <c r="E5" s="213"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -4134,10 +4143,10 @@
         <v>72</v>
       </c>
       <c r="C6" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="34" t="s">
         <v>148</v>
-      </c>
-      <c r="D6" s="34" t="s">
-        <v>149</v>
       </c>
       <c r="E6" s="35" t="s">
         <v>73</v>
@@ -4173,27 +4182,27 @@
         <v>76</v>
       </c>
       <c r="C7" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="D7" s="34" t="s">
         <v>150</v>
-      </c>
-      <c r="D7" s="34" t="s">
-        <v>151</v>
       </c>
       <c r="E7" s="34" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:26">
-      <c r="A8" s="218">
+      <c r="A8" s="212">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B8" s="228" t="s">
+      <c r="B8" s="219" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="229" t="s">
-        <v>152</v>
-      </c>
-      <c r="D8" s="230" t="s">
+      <c r="C8" s="220" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8" s="221" t="s">
         <v>35</v>
       </c>
       <c r="E8" s="36" t="s">
@@ -4222,10 +4231,10 @@
       <c r="Z8" s="11"/>
     </row>
     <row r="9" spans="1:26">
-      <c r="A9" s="234"/>
-      <c r="B9" s="235"/>
-      <c r="C9" s="236"/>
-      <c r="D9" s="234"/>
+      <c r="A9" s="213"/>
+      <c r="B9" s="215"/>
+      <c r="C9" s="217"/>
+      <c r="D9" s="213"/>
       <c r="E9" s="36" t="s">
         <v>37</v>
       </c>
@@ -4252,17 +4261,17 @@
       <c r="Z9" s="11"/>
     </row>
     <row r="10" spans="1:26">
-      <c r="A10" s="210">
+      <c r="A10" s="224">
         <f>SUM(A8+1)</f>
         <v>6</v>
       </c>
-      <c r="B10" s="220" t="s">
+      <c r="B10" s="225" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="221" t="s">
-        <v>153</v>
-      </c>
-      <c r="D10" s="209" t="s">
+      <c r="C10" s="226" t="s">
+        <v>152</v>
+      </c>
+      <c r="D10" s="227" t="s">
         <v>40</v>
       </c>
       <c r="E10" s="34" t="s">
@@ -4291,10 +4300,10 @@
       <c r="Z10" s="13"/>
     </row>
     <row r="11" spans="1:26">
-      <c r="A11" s="234"/>
-      <c r="B11" s="235"/>
-      <c r="C11" s="236"/>
-      <c r="D11" s="234"/>
+      <c r="A11" s="213"/>
+      <c r="B11" s="215"/>
+      <c r="C11" s="217"/>
+      <c r="D11" s="213"/>
       <c r="E11" s="34" t="s">
         <v>41</v>
       </c>
@@ -4321,21 +4330,21 @@
       <c r="Z11" s="13"/>
     </row>
     <row r="12" spans="1:26">
-      <c r="A12" s="224">
+      <c r="A12" s="228">
         <f>SUM(A10+1)</f>
         <v>7</v>
       </c>
-      <c r="B12" s="225" t="s">
+      <c r="B12" s="229" t="s">
+        <v>153</v>
+      </c>
+      <c r="C12" s="222" t="s">
         <v>154</v>
       </c>
-      <c r="C12" s="222" t="s">
+      <c r="D12" s="223" t="s">
         <v>155</v>
       </c>
-      <c r="D12" s="223" t="s">
+      <c r="E12" s="14" t="s">
         <v>156</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>157</v>
       </c>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
@@ -4360,12 +4369,12 @@
       <c r="Z12" s="15"/>
     </row>
     <row r="13" spans="1:26">
-      <c r="A13" s="234"/>
-      <c r="B13" s="235"/>
-      <c r="C13" s="236"/>
-      <c r="D13" s="234"/>
+      <c r="A13" s="213"/>
+      <c r="B13" s="215"/>
+      <c r="C13" s="217"/>
+      <c r="D13" s="213"/>
       <c r="E13" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
@@ -4390,15 +4399,15 @@
       <c r="Z13" s="15"/>
     </row>
     <row r="14" spans="1:26">
-      <c r="A14" s="210">
+      <c r="A14" s="224">
         <f>SUM(A12+1)</f>
         <v>8</v>
       </c>
-      <c r="B14" s="220" t="s">
+      <c r="B14" s="225" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="221" t="s">
-        <v>159</v>
+      <c r="C14" s="226" t="s">
+        <v>158</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>46</v>
@@ -4408,14 +4417,14 @@
       </c>
     </row>
     <row r="15" spans="1:26">
-      <c r="A15" s="234"/>
-      <c r="B15" s="235"/>
-      <c r="C15" s="236"/>
+      <c r="A15" s="213"/>
+      <c r="B15" s="215"/>
+      <c r="C15" s="217"/>
       <c r="D15" s="34" t="s">
         <v>49</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:26">
@@ -4427,7 +4436,7 @@
         <v>56</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D16" s="36" t="s">
         <v>61</v>
@@ -4458,17 +4467,17 @@
       <c r="Z16" s="11"/>
     </row>
     <row r="17" spans="1:26">
-      <c r="A17" s="210">
+      <c r="A17" s="224">
         <f>A16+1</f>
         <v>10</v>
       </c>
       <c r="B17" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="215" t="s">
-        <v>162</v>
-      </c>
-      <c r="D17" s="209" t="s">
+      <c r="C17" s="230" t="s">
+        <v>161</v>
+      </c>
+      <c r="D17" s="227" t="s">
         <v>68</v>
       </c>
       <c r="E17" s="34" t="s">
@@ -4497,14 +4506,14 @@
       <c r="Z17" s="18"/>
     </row>
     <row r="18" spans="1:26">
-      <c r="A18" s="234"/>
+      <c r="A18" s="213"/>
       <c r="B18" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="236"/>
-      <c r="D18" s="234"/>
+      <c r="C18" s="217"/>
+      <c r="D18" s="213"/>
       <c r="E18" s="34" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F18" s="18"/>
       <c r="G18" s="18"/>
@@ -4528,7 +4537,7 @@
       <c r="Y18" s="18"/>
       <c r="Z18" s="18"/>
     </row>
-    <row r="19" spans="1:26" ht="15.95">
+    <row r="19" spans="1:26" ht="16">
       <c r="A19" s="16">
         <f>A17+1</f>
         <v>11</v>
@@ -4537,7 +4546,7 @@
         <v>92</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D19" s="41" t="s">
         <v>94</v>
@@ -4567,19 +4576,19 @@
       <c r="Y19" s="11"/>
       <c r="Z19" s="11"/>
     </row>
-    <row r="20" spans="1:26" ht="15.95">
+    <row r="20" spans="1:26" ht="16">
       <c r="A20" s="19">
         <f t="shared" ref="A20:A21" si="1">A19+1</f>
         <v>12</v>
       </c>
       <c r="B20" s="43" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="44" t="s">
         <v>165</v>
       </c>
-      <c r="C20" s="44" t="s">
+      <c r="D20" s="20" t="s">
         <v>166</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>167</v>
       </c>
       <c r="E20" s="21"/>
       <c r="F20" s="22"/>
@@ -4613,7 +4622,7 @@
         <v>15</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D21" s="46" t="s">
         <v>16</v>
@@ -4626,10 +4635,10 @@
         <v>14</v>
       </c>
       <c r="B22" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="C22" s="33" t="s">
         <v>169</v>
-      </c>
-      <c r="C22" s="33" t="s">
-        <v>170</v>
       </c>
       <c r="D22" s="34" t="s">
         <v>87</v>
@@ -4665,13 +4674,13 @@
         <v>15</v>
       </c>
       <c r="B23" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="C23" s="52" t="s">
         <v>171</v>
       </c>
-      <c r="C23" s="52" t="s">
+      <c r="D23" s="29" t="s">
         <v>172</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>173</v>
       </c>
       <c r="E23" s="53"/>
     </row>
@@ -4681,13 +4690,13 @@
         <v>16</v>
       </c>
       <c r="B24" s="47" t="s">
+        <v>173</v>
+      </c>
+      <c r="C24" s="54" t="s">
+        <v>167</v>
+      </c>
+      <c r="D24" s="55" t="s">
         <v>174</v>
-      </c>
-      <c r="C24" s="54" t="s">
-        <v>168</v>
-      </c>
-      <c r="D24" s="55" t="s">
-        <v>175</v>
       </c>
       <c r="E24" s="56"/>
       <c r="F24" s="11"/>
@@ -4713,18 +4722,18 @@
       <c r="Z24" s="11"/>
     </row>
     <row r="25" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A25" s="210">
+      <c r="A25" s="224">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="B25" s="214" t="s">
-        <v>106</v>
-      </c>
-      <c r="C25" s="215" t="s">
-        <v>176</v>
-      </c>
-      <c r="D25" s="211" t="s">
-        <v>109</v>
+      <c r="B25" s="234" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="230" t="s">
+        <v>175</v>
+      </c>
+      <c r="D25" s="231" t="s">
+        <v>108</v>
       </c>
       <c r="E25" s="35" t="s">
         <v>91</v>
@@ -4752,12 +4761,12 @@
       <c r="Z25" s="24"/>
     </row>
     <row r="26" spans="1:26" ht="15" customHeight="1">
-      <c r="A26" s="234"/>
-      <c r="B26" s="235"/>
-      <c r="C26" s="236"/>
-      <c r="D26" s="234"/>
+      <c r="A26" s="213"/>
+      <c r="B26" s="215"/>
+      <c r="C26" s="217"/>
+      <c r="D26" s="213"/>
       <c r="E26" s="34" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F26" s="24"/>
       <c r="G26" s="24"/>
@@ -4787,13 +4796,13 @@
         <v>18</v>
       </c>
       <c r="B27" s="48" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E27" s="26"/>
       <c r="F27" s="11"/>
@@ -4819,21 +4828,21 @@
       <c r="Z27" s="11"/>
     </row>
     <row r="28" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A28" s="216">
+      <c r="A28" s="235">
         <f>A27+1</f>
         <v>19</v>
       </c>
-      <c r="B28" s="217" t="s">
-        <v>132</v>
-      </c>
-      <c r="C28" s="215" t="s">
-        <v>178</v>
-      </c>
-      <c r="D28" s="209" t="s">
+      <c r="B28" s="236" t="s">
+        <v>131</v>
+      </c>
+      <c r="C28" s="230" t="s">
+        <v>177</v>
+      </c>
+      <c r="D28" s="227" t="s">
+        <v>129</v>
+      </c>
+      <c r="E28" s="34" t="s">
         <v>130</v>
-      </c>
-      <c r="E28" s="34" t="s">
-        <v>131</v>
       </c>
       <c r="F28" s="10"/>
       <c r="G28" s="10"/>
@@ -4858,12 +4867,12 @@
       <c r="Z28" s="10"/>
     </row>
     <row r="29" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A29" s="234"/>
-      <c r="B29" s="235"/>
-      <c r="C29" s="236"/>
-      <c r="D29" s="234"/>
+      <c r="A29" s="213"/>
+      <c r="B29" s="215"/>
+      <c r="C29" s="217"/>
+      <c r="D29" s="213"/>
       <c r="E29" s="34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
@@ -4888,21 +4897,21 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A30" s="218">
+      <c r="A30" s="212">
         <f>A28+1</f>
         <v>20</v>
       </c>
-      <c r="B30" s="212" t="s">
-        <v>135</v>
-      </c>
-      <c r="C30" s="213" t="s">
+      <c r="B30" s="232" t="s">
+        <v>134</v>
+      </c>
+      <c r="C30" s="233" t="s">
+        <v>178</v>
+      </c>
+      <c r="D30" s="218" t="s">
         <v>179</v>
       </c>
-      <c r="D30" s="219" t="s">
-        <v>180</v>
-      </c>
       <c r="E30" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F30" s="11"/>
       <c r="G30" s="11"/>
@@ -4927,12 +4936,12 @@
       <c r="Z30" s="11"/>
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A31" s="234"/>
-      <c r="B31" s="235"/>
-      <c r="C31" s="236"/>
-      <c r="D31" s="234"/>
+      <c r="A31" s="213"/>
+      <c r="B31" s="215"/>
+      <c r="C31" s="217"/>
+      <c r="D31" s="213"/>
       <c r="E31" s="41" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F31" s="11"/>
       <c r="G31" s="11"/>
@@ -4962,13 +4971,13 @@
         <v>21</v>
       </c>
       <c r="B32" s="45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D32" s="35" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E32" s="27"/>
     </row>
@@ -4978,13 +4987,13 @@
         <v>22</v>
       </c>
       <c r="B33" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="D33" s="34" t="s">
         <v>119</v>
-      </c>
-      <c r="C33" s="33" t="s">
-        <v>182</v>
-      </c>
-      <c r="D33" s="34" t="s">
-        <v>120</v>
       </c>
       <c r="E33" s="27"/>
       <c r="F33" s="24"/>
@@ -5015,14 +5024,14 @@
         <v>24</v>
       </c>
       <c r="B34" s="41" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D34" s="41"/>
       <c r="E34" s="36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F34" s="11"/>
       <c r="G34" s="11"/>
@@ -11810,27 +11819,6 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="C17:C18"/>
     <mergeCell ref="D17:D18"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="D25:D26"/>
@@ -11844,6 +11832,27 @@
     <mergeCell ref="D28:D29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="D30:D31"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
@@ -11934,17 +11943,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f0b0792d-d654-4f32-9135-0cf693c22f67">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c805177d-b823-4c7f-87f1-c3fe271a3d2d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD90A491793F574D833EEF3FF0869CA1" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b15b8ac1b6df1795c032a72689c8e15f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f0b0792d-d654-4f32-9135-0cf693c22f67" xmlns:ns3="c805177d-b823-4c7f-87f1-c3fe271a3d2d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7e45a94f909e329f9a8ac4529b6db8ce" ns2:_="" ns3:_="">
     <xsd:import namespace="f0b0792d-d654-4f32-9135-0cf693c22f67"/>
@@ -12199,16 +12197,53 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f0b0792d-d654-4f32-9135-0cf693c22f67">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c805177d-b823-4c7f-87f1-c3fe271a3d2d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1393095-9EBA-4193-AB4B-17269DE767FD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1393095-9EBA-4193-AB4B-17269DE767FD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E1BC49D-499B-4FD5-B4A6-90CBD04CEF93}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{451CC68B-C786-4554-BF8A-BED96CCD5B5C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f0b0792d-d654-4f32-9135-0cf693c22f67"/>
+    <ds:schemaRef ds:uri="c805177d-b823-4c7f-87f1-c3fe271a3d2d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{451CC68B-C786-4554-BF8A-BED96CCD5B5C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E1BC49D-499B-4FD5-B4A6-90CBD04CEF93}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f0b0792d-d654-4f32-9135-0cf693c22f67"/>
+    <ds:schemaRef ds:uri="c805177d-b823-4c7f-87f1-c3fe271a3d2d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Fix typo in spreadsheet (#11)
* Fix typo in spreadsheet

* Fix typo: "Provanance" → "Provenance" in row 15 topic column
</commit_message>
<xml_diff>
--- a/docs/CS858-F26-papers-stripped.xlsx
+++ b/docs/CS858-F26-papers-stripped.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uofwaterloo.sharepoint.com/sites/tm-math-ssg-mlsec/Shared Documents/General/MLSec-tutorial/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/asimwaheed/Documents/AllWork/Bots/cs858-wiki/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="660" documentId="11_A6B81843C1AE8CB9D7F3088654DFBA397E707E1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5268A3D0-5EBE-4472-B911-E35DA6356959}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F676B01-4AA7-264A-A01E-1318C8A08329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33420" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="33420" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UpdatedList" sheetId="1" r:id="rId1"/>
@@ -344,9 +344,6 @@
     <t>A Watermark for Large Language Models</t>
   </si>
   <si>
-    <t>Media Forensics and Proactive Provanance</t>
-  </si>
-  <si>
     <t>Tree-Ring Watermarks: Fingerprints for Diffusion Images that are Invisible and Robust</t>
   </si>
   <si>
@@ -616,12 +613,15 @@
   <si>
     <t>Model Theft Resistance (+ on-device private inference)  - Hardware</t>
   </si>
+  <si>
+    <t>Media Forensics and Proactive Provenance</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="38">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -847,6 +847,12 @@
     <font>
       <sz val="12"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1131,7 +1137,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="237">
+  <cellXfs count="238">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1431,24 +1437,219 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="7" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="7" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1473,203 +1674,56 @@
     <xf numFmtId="0" fontId="34" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
@@ -1683,60 +1737,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1963,16 +1972,16 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AB51"/>
-  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" style="31"/>
-    <col min="2" max="2" width="100.42578125" style="67" customWidth="1"/>
-    <col min="3" max="3" width="52.140625" style="67" customWidth="1"/>
-    <col min="4" max="4" width="40.7109375" style="31" customWidth="1"/>
-    <col min="5" max="5" width="90.85546875" style="31" customWidth="1"/>
+    <col min="1" max="1" width="12.5" style="31"/>
+    <col min="2" max="2" width="100.5" style="67" customWidth="1"/>
+    <col min="3" max="3" width="52.1640625" style="67" customWidth="1"/>
+    <col min="4" max="4" width="40.6640625" style="31" customWidth="1"/>
+    <col min="5" max="5" width="90.83203125" style="31" customWidth="1"/>
     <col min="6" max="6" width="72" style="31" customWidth="1"/>
-    <col min="7" max="7" width="83.42578125" style="31" customWidth="1"/>
-    <col min="8" max="16384" width="12.42578125" style="31"/>
+    <col min="7" max="7" width="83.5" style="31" customWidth="1"/>
+    <col min="8" max="16384" width="12.5" style="31"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="15" customHeight="1">
@@ -1997,34 +2006,34 @@
       </c>
     </row>
     <row r="2" spans="1:28" s="79" customFormat="1" ht="15" customHeight="1">
-      <c r="A2" s="169" t="s">
+      <c r="A2" s="172" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="170"/>
-      <c r="C2" s="170"/>
-      <c r="D2" s="170"/>
-      <c r="E2" s="171"/>
+      <c r="B2" s="173"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="174"/>
       <c r="F2" s="59"/>
       <c r="G2" s="78"/>
     </row>
     <row r="3" spans="1:28" ht="15" customHeight="1">
-      <c r="A3" s="154">
+      <c r="A3" s="133">
         <v>1</v>
       </c>
-      <c r="B3" s="208" t="s">
+      <c r="B3" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="180" t="s">
+      <c r="C3" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="154" t="s">
+      <c r="D3" s="133" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="104" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="59"/>
-      <c r="G3" s="205" t="s">
+      <c r="G3" s="131" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="80"/>
@@ -2050,15 +2059,15 @@
       <c r="AB3" s="80"/>
     </row>
     <row r="4" spans="1:28" ht="15" customHeight="1">
-      <c r="A4" s="231"/>
-      <c r="B4" s="208"/>
-      <c r="C4" s="181"/>
-      <c r="D4" s="231"/>
+      <c r="A4" s="134"/>
+      <c r="B4" s="144"/>
+      <c r="C4" s="161"/>
+      <c r="D4" s="134"/>
       <c r="E4" s="105" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="59"/>
-      <c r="G4" s="232"/>
+      <c r="G4" s="132"/>
       <c r="H4" s="80"/>
       <c r="I4" s="80"/>
       <c r="J4" s="80"/>
@@ -2082,14 +2091,14 @@
       <c r="AB4" s="80"/>
     </row>
     <row r="5" spans="1:28" ht="15" customHeight="1">
-      <c r="A5" s="154">
+      <c r="A5" s="133">
         <v>2</v>
       </c>
-      <c r="B5" s="178" t="s">
+      <c r="B5" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="181"/>
-      <c r="D5" s="154" t="s">
+      <c r="C5" s="161"/>
+      <c r="D5" s="133" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="104" t="s">
@@ -2124,10 +2133,10 @@
       <c r="AB5" s="30"/>
     </row>
     <row r="6" spans="1:28" ht="15" customHeight="1">
-      <c r="A6" s="231"/>
-      <c r="B6" s="179"/>
-      <c r="C6" s="181"/>
-      <c r="D6" s="231"/>
+      <c r="A6" s="134"/>
+      <c r="B6" s="146"/>
+      <c r="C6" s="161"/>
+      <c r="D6" s="134"/>
       <c r="E6" s="105" t="s">
         <v>18</v>
       </c>
@@ -2158,14 +2167,14 @@
       <c r="AB6" s="30"/>
     </row>
     <row r="7" spans="1:28" ht="15" customHeight="1">
-      <c r="A7" s="154">
+      <c r="A7" s="133">
         <v>3</v>
       </c>
-      <c r="B7" s="178" t="s">
+      <c r="B7" s="145" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="181"/>
-      <c r="D7" s="154" t="s">
+      <c r="C7" s="161"/>
+      <c r="D7" s="133" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="104" t="s">
@@ -2196,10 +2205,10 @@
       <c r="AB7" s="30"/>
     </row>
     <row r="8" spans="1:28" ht="15" customHeight="1">
-      <c r="A8" s="231"/>
-      <c r="B8" s="179"/>
-      <c r="C8" s="181"/>
-      <c r="D8" s="231"/>
+      <c r="A8" s="134"/>
+      <c r="B8" s="146"/>
+      <c r="C8" s="161"/>
+      <c r="D8" s="134"/>
       <c r="E8" s="106" t="s">
         <v>23</v>
       </c>
@@ -2228,14 +2237,14 @@
       <c r="AB8" s="30"/>
     </row>
     <row r="9" spans="1:28" ht="15" customHeight="1">
-      <c r="A9" s="154">
+      <c r="A9" s="133">
         <v>4</v>
       </c>
-      <c r="B9" s="203" t="s">
+      <c r="B9" s="137" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="181"/>
-      <c r="D9" s="154" t="s">
+      <c r="C9" s="161"/>
+      <c r="D9" s="133" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="104" t="s">
@@ -2270,10 +2279,10 @@
       <c r="AB9" s="30"/>
     </row>
     <row r="10" spans="1:28" ht="15" customHeight="1">
-      <c r="A10" s="231"/>
-      <c r="B10" s="204"/>
-      <c r="C10" s="182"/>
-      <c r="D10" s="231"/>
+      <c r="A10" s="134"/>
+      <c r="B10" s="138"/>
+      <c r="C10" s="162"/>
+      <c r="D10" s="134"/>
       <c r="E10" s="106" t="s">
         <v>29</v>
       </c>
@@ -2304,16 +2313,16 @@
       <c r="AB10" s="30"/>
     </row>
     <row r="11" spans="1:28" ht="15" customHeight="1">
-      <c r="A11" s="145">
+      <c r="A11" s="135">
         <v>5</v>
       </c>
-      <c r="B11" s="201" t="s">
+      <c r="B11" s="139" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="189" t="s">
+      <c r="C11" s="154" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="149" t="s">
+      <c r="D11" s="143" t="s">
         <v>33</v>
       </c>
       <c r="E11" s="107" t="s">
@@ -2346,10 +2355,10 @@
       <c r="AB11" s="30"/>
     </row>
     <row r="12" spans="1:28" ht="15" customHeight="1">
-      <c r="A12" s="233"/>
-      <c r="B12" s="202"/>
-      <c r="C12" s="190"/>
-      <c r="D12" s="233"/>
+      <c r="A12" s="136"/>
+      <c r="B12" s="140"/>
+      <c r="C12" s="155"/>
+      <c r="D12" s="136"/>
       <c r="E12" s="108" t="s">
         <v>36</v>
       </c>
@@ -2380,14 +2389,14 @@
       <c r="AB12" s="30"/>
     </row>
     <row r="13" spans="1:28" ht="15" customHeight="1">
-      <c r="A13" s="145">
+      <c r="A13" s="135">
         <v>6</v>
       </c>
-      <c r="B13" s="201" t="s">
+      <c r="B13" s="139" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="190"/>
-      <c r="D13" s="149" t="s">
+      <c r="C13" s="155"/>
+      <c r="D13" s="143" t="s">
         <v>39</v>
       </c>
       <c r="E13" s="109" t="s">
@@ -2420,10 +2429,10 @@
       <c r="AB13" s="30"/>
     </row>
     <row r="14" spans="1:28" ht="15" customHeight="1">
-      <c r="A14" s="233"/>
-      <c r="B14" s="202"/>
-      <c r="C14" s="190"/>
-      <c r="D14" s="233"/>
+      <c r="A14" s="136"/>
+      <c r="B14" s="140"/>
+      <c r="C14" s="155"/>
+      <c r="D14" s="136"/>
       <c r="E14" s="108" t="s">
         <v>42</v>
       </c>
@@ -2454,14 +2463,14 @@
       <c r="AB14" s="30"/>
     </row>
     <row r="15" spans="1:28" ht="15" customHeight="1">
-      <c r="A15" s="145">
+      <c r="A15" s="135">
         <v>7</v>
       </c>
-      <c r="B15" s="201" t="s">
+      <c r="B15" s="139" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="190"/>
-      <c r="D15" s="149" t="s">
+      <c r="C15" s="155"/>
+      <c r="D15" s="143" t="s">
         <v>45</v>
       </c>
       <c r="E15" s="110" t="s">
@@ -2494,10 +2503,10 @@
       <c r="AB15" s="30"/>
     </row>
     <row r="16" spans="1:28" ht="15" customHeight="1">
-      <c r="A16" s="233"/>
-      <c r="B16" s="202"/>
-      <c r="C16" s="190"/>
-      <c r="D16" s="233"/>
+      <c r="A16" s="136"/>
+      <c r="B16" s="140"/>
+      <c r="C16" s="155"/>
+      <c r="D16" s="136"/>
       <c r="E16" s="108" t="s">
         <v>48</v>
       </c>
@@ -2528,14 +2537,14 @@
       <c r="AB16" s="30"/>
     </row>
     <row r="17" spans="1:28" ht="15" customHeight="1">
-      <c r="A17" s="145">
+      <c r="A17" s="135">
         <v>8</v>
       </c>
-      <c r="B17" s="176" t="s">
+      <c r="B17" s="178" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="190"/>
-      <c r="D17" s="145" t="s">
+      <c r="C17" s="155"/>
+      <c r="D17" s="135" t="s">
         <v>51</v>
       </c>
       <c r="E17" s="110" t="s">
@@ -2567,10 +2576,10 @@
       <c r="AB17" s="30"/>
     </row>
     <row r="18" spans="1:28" ht="15" customHeight="1">
-      <c r="A18" s="233"/>
-      <c r="B18" s="177"/>
-      <c r="C18" s="191"/>
-      <c r="D18" s="233"/>
+      <c r="A18" s="136"/>
+      <c r="B18" s="179"/>
+      <c r="C18" s="156"/>
+      <c r="D18" s="136"/>
       <c r="E18" s="111" t="s">
         <v>54</v>
       </c>
@@ -2603,16 +2612,16 @@
       <c r="AB18" s="30"/>
     </row>
     <row r="19" spans="1:28" ht="15" customHeight="1">
-      <c r="A19" s="154">
+      <c r="A19" s="133">
         <v>9</v>
       </c>
-      <c r="B19" s="178" t="s">
+      <c r="B19" s="145" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="192" t="s">
+      <c r="C19" s="157" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="154" t="s">
+      <c r="D19" s="133" t="s">
         <v>58</v>
       </c>
       <c r="E19" s="104" t="s">
@@ -2645,10 +2654,10 @@
       <c r="AB19" s="30"/>
     </row>
     <row r="20" spans="1:28" ht="15" customHeight="1">
-      <c r="A20" s="231"/>
-      <c r="B20" s="179"/>
-      <c r="C20" s="193"/>
-      <c r="D20" s="231"/>
+      <c r="A20" s="134"/>
+      <c r="B20" s="146"/>
+      <c r="C20" s="158"/>
+      <c r="D20" s="134"/>
       <c r="E20" s="105" t="s">
         <v>61</v>
       </c>
@@ -2679,14 +2688,14 @@
       <c r="AB20" s="30"/>
     </row>
     <row r="21" spans="1:28" ht="15" customHeight="1">
-      <c r="A21" s="154">
+      <c r="A21" s="133">
         <v>10</v>
       </c>
-      <c r="B21" s="178" t="s">
+      <c r="B21" s="145" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="193"/>
-      <c r="D21" s="175" t="s">
+      <c r="C21" s="158"/>
+      <c r="D21" s="170" t="s">
         <v>64</v>
       </c>
       <c r="E21" s="104" t="s">
@@ -2719,10 +2728,10 @@
       <c r="AB21" s="30"/>
     </row>
     <row r="22" spans="1:28" ht="15" customHeight="1">
-      <c r="A22" s="231"/>
-      <c r="B22" s="179"/>
-      <c r="C22" s="194"/>
-      <c r="D22" s="231"/>
+      <c r="A22" s="134"/>
+      <c r="B22" s="146"/>
+      <c r="C22" s="159"/>
+      <c r="D22" s="134"/>
       <c r="E22" s="112" t="s">
         <v>67</v>
       </c>
@@ -2753,16 +2762,16 @@
       <c r="AB22" s="30"/>
     </row>
     <row r="23" spans="1:28" ht="15" customHeight="1">
-      <c r="A23" s="145">
+      <c r="A23" s="135">
         <v>11</v>
       </c>
-      <c r="B23" s="206" t="s">
+      <c r="B23" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="195" t="s">
+      <c r="C23" s="147" t="s">
         <v>70</v>
       </c>
-      <c r="D23" s="145" t="s">
+      <c r="D23" s="135" t="s">
         <v>71</v>
       </c>
       <c r="E23" s="110" t="s">
@@ -2796,10 +2805,10 @@
       <c r="AB23" s="80"/>
     </row>
     <row r="24" spans="1:28" ht="15" customHeight="1">
-      <c r="A24" s="233"/>
-      <c r="B24" s="207"/>
-      <c r="C24" s="196"/>
-      <c r="D24" s="233"/>
+      <c r="A24" s="136"/>
+      <c r="B24" s="142"/>
+      <c r="C24" s="148"/>
+      <c r="D24" s="136"/>
       <c r="E24" s="108" t="s">
         <v>75</v>
       </c>
@@ -2832,14 +2841,14 @@
       <c r="AB24" s="80"/>
     </row>
     <row r="25" spans="1:28" ht="15" customHeight="1">
-      <c r="A25" s="145">
+      <c r="A25" s="135">
         <v>12</v>
       </c>
-      <c r="B25" s="206" t="s">
+      <c r="B25" s="141" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="196"/>
-      <c r="D25" s="145" t="s">
+      <c r="C25" s="148"/>
+      <c r="D25" s="135" t="s">
         <v>79</v>
       </c>
       <c r="E25" s="110" t="s">
@@ -2869,10 +2878,10 @@
       <c r="AB25" s="30"/>
     </row>
     <row r="26" spans="1:28" ht="15" customHeight="1">
-      <c r="A26" s="233"/>
-      <c r="B26" s="207"/>
-      <c r="C26" s="197"/>
-      <c r="D26" s="233"/>
+      <c r="A26" s="136"/>
+      <c r="B26" s="142"/>
+      <c r="C26" s="149"/>
+      <c r="D26" s="136"/>
       <c r="E26" s="108" t="s">
         <v>81</v>
       </c>
@@ -2903,16 +2912,16 @@
       <c r="AB26" s="30"/>
     </row>
     <row r="27" spans="1:28" ht="15" customHeight="1">
-      <c r="A27" s="154">
+      <c r="A27" s="133">
         <v>13</v>
       </c>
-      <c r="B27" s="203" t="s">
+      <c r="B27" s="137" t="s">
         <v>83</v>
       </c>
-      <c r="C27" s="198" t="s">
+      <c r="C27" s="150" t="s">
         <v>84</v>
       </c>
-      <c r="D27" s="154" t="s">
+      <c r="D27" s="133" t="s">
         <v>85</v>
       </c>
       <c r="E27" s="104" t="s">
@@ -2949,10 +2958,10 @@
       <c r="AB27" s="30"/>
     </row>
     <row r="28" spans="1:28" ht="15" customHeight="1">
-      <c r="A28" s="231"/>
-      <c r="B28" s="204"/>
-      <c r="C28" s="199"/>
-      <c r="D28" s="155"/>
+      <c r="A28" s="134"/>
+      <c r="B28" s="138"/>
+      <c r="C28" s="151"/>
+      <c r="D28" s="153"/>
       <c r="E28" s="113" t="s">
         <v>90</v>
       </c>
@@ -2982,14 +2991,14 @@
       <c r="AB28" s="30"/>
     </row>
     <row r="29" spans="1:28" ht="15" customHeight="1">
-      <c r="A29" s="154">
+      <c r="A29" s="133">
         <v>14</v>
       </c>
-      <c r="B29" s="178" t="s">
+      <c r="B29" s="145" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="199"/>
-      <c r="D29" s="154" t="s">
+      <c r="C29" s="151"/>
+      <c r="D29" s="133" t="s">
         <v>93</v>
       </c>
       <c r="E29" s="104" t="s">
@@ -3020,10 +3029,10 @@
       <c r="AB29" s="30"/>
     </row>
     <row r="30" spans="1:28" ht="15" customHeight="1">
-      <c r="A30" s="231"/>
-      <c r="B30" s="179"/>
-      <c r="C30" s="199"/>
-      <c r="D30" s="155"/>
+      <c r="A30" s="134"/>
+      <c r="B30" s="146"/>
+      <c r="C30" s="151"/>
+      <c r="D30" s="153"/>
       <c r="E30" s="105" t="s">
         <v>95</v>
       </c>
@@ -3051,46 +3060,46 @@
       <c r="AB30" s="30"/>
     </row>
     <row r="31" spans="1:28" ht="15" customHeight="1">
-      <c r="A31" s="154">
+      <c r="A31" s="133">
         <v>15</v>
       </c>
-      <c r="B31" s="203" t="s">
+      <c r="B31" s="137" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="199"/>
-      <c r="D31" s="154" t="s">
+      <c r="C31" s="151"/>
+      <c r="D31" s="237" t="s">
+        <v>183</v>
+      </c>
+      <c r="E31" s="114" t="s">
         <v>97</v>
-      </c>
-      <c r="E31" s="114" t="s">
-        <v>98</v>
       </c>
       <c r="F31" s="63"/>
       <c r="G31" s="70"/>
     </row>
     <row r="32" spans="1:28" ht="15" customHeight="1">
-      <c r="A32" s="231"/>
-      <c r="B32" s="204"/>
-      <c r="C32" s="199"/>
-      <c r="D32" s="155"/>
+      <c r="A32" s="134"/>
+      <c r="B32" s="138"/>
+      <c r="C32" s="151"/>
+      <c r="D32" s="153"/>
       <c r="E32" s="115" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F32" s="59"/>
       <c r="G32" s="70"/>
     </row>
     <row r="33" spans="1:28" ht="15" customHeight="1">
-      <c r="A33" s="154">
+      <c r="A33" s="133">
         <v>16</v>
       </c>
-      <c r="B33" s="178" t="s">
+      <c r="B33" s="145" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="151"/>
+      <c r="D33" s="133" t="s">
         <v>100</v>
       </c>
-      <c r="C33" s="199"/>
-      <c r="D33" s="154" t="s">
+      <c r="E33" s="104" t="s">
         <v>101</v>
-      </c>
-      <c r="E33" s="104" t="s">
-        <v>102</v>
       </c>
       <c r="F33" s="59"/>
       <c r="H33" s="30"/>
@@ -3116,16 +3125,16 @@
       <c r="AB33" s="30"/>
     </row>
     <row r="34" spans="1:28" ht="15" customHeight="1">
-      <c r="A34" s="231"/>
-      <c r="B34" s="179"/>
-      <c r="C34" s="200"/>
-      <c r="D34" s="231"/>
+      <c r="A34" s="134"/>
+      <c r="B34" s="146"/>
+      <c r="C34" s="152"/>
+      <c r="D34" s="134"/>
       <c r="E34" s="113" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F34" s="64"/>
       <c r="G34" s="71" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H34" s="30"/>
       <c r="I34" s="30"/>
@@ -3150,13 +3159,13 @@
       <c r="AB34" s="30"/>
     </row>
     <row r="35" spans="1:28" ht="15" customHeight="1">
-      <c r="A35" s="172" t="s">
-        <v>105</v>
-      </c>
-      <c r="B35" s="173"/>
-      <c r="C35" s="173"/>
-      <c r="D35" s="173"/>
-      <c r="E35" s="174"/>
+      <c r="A35" s="175" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" s="176"/>
+      <c r="C35" s="176"/>
+      <c r="D35" s="176"/>
+      <c r="E35" s="177"/>
       <c r="F35" s="72"/>
       <c r="G35" s="73"/>
       <c r="H35" s="30"/>
@@ -3182,20 +3191,20 @@
       <c r="AB35" s="30"/>
     </row>
     <row r="36" spans="1:28" ht="15" customHeight="1">
-      <c r="A36" s="154">
+      <c r="A36" s="133">
         <v>17</v>
       </c>
-      <c r="B36" s="186" t="s">
+      <c r="B36" s="168" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" s="184" t="s">
         <v>106</v>
       </c>
-      <c r="C36" s="151" t="s">
+      <c r="D36" s="170" t="s">
         <v>107</v>
       </c>
-      <c r="D36" s="175" t="s">
+      <c r="E36" s="116" t="s">
         <v>108</v>
-      </c>
-      <c r="E36" s="116" t="s">
-        <v>109</v>
       </c>
       <c r="F36" s="74"/>
       <c r="G36" s="72" t="s">
@@ -3224,14 +3233,14 @@
       <c r="AB36" s="30"/>
     </row>
     <row r="37" spans="1:28" ht="15" customHeight="1">
-      <c r="A37" s="161"/>
-      <c r="B37" s="187"/>
-      <c r="C37" s="152"/>
-      <c r="D37" s="188"/>
+      <c r="A37" s="192"/>
+      <c r="B37" s="169"/>
+      <c r="C37" s="185"/>
+      <c r="D37" s="171"/>
       <c r="E37" s="117"/>
       <c r="F37" s="58"/>
       <c r="G37" s="75" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H37" s="30"/>
       <c r="I37" s="30"/>
@@ -3256,18 +3265,18 @@
       <c r="AB37" s="30"/>
     </row>
     <row r="38" spans="1:28" ht="15" customHeight="1">
-      <c r="A38" s="154">
+      <c r="A38" s="133">
         <v>18</v>
       </c>
-      <c r="B38" s="156" t="s">
+      <c r="B38" s="187" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" s="185"/>
+      <c r="D38" s="133" t="s">
         <v>111</v>
       </c>
-      <c r="C38" s="152"/>
-      <c r="D38" s="154" t="s">
+      <c r="E38" s="118" t="s">
         <v>112</v>
-      </c>
-      <c r="E38" s="118" t="s">
-        <v>113</v>
       </c>
       <c r="F38" s="58"/>
       <c r="G38" s="75"/>
@@ -3294,10 +3303,10 @@
       <c r="AB38" s="30"/>
     </row>
     <row r="39" spans="1:28" ht="15" customHeight="1">
-      <c r="A39" s="155"/>
-      <c r="B39" s="157"/>
-      <c r="C39" s="153"/>
-      <c r="D39" s="155"/>
+      <c r="A39" s="153"/>
+      <c r="B39" s="188"/>
+      <c r="C39" s="186"/>
+      <c r="D39" s="153"/>
       <c r="E39" s="119"/>
       <c r="F39" s="75"/>
       <c r="G39" s="76"/>
@@ -3324,24 +3333,24 @@
       <c r="AB39" s="30"/>
     </row>
     <row r="40" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A40" s="135">
+      <c r="A40" s="163">
         <v>19</v>
       </c>
-      <c r="B40" s="184" t="s">
+      <c r="B40" s="165" t="s">
+        <v>113</v>
+      </c>
+      <c r="C40" s="206" t="s">
         <v>114</v>
       </c>
-      <c r="C40" s="139" t="s">
+      <c r="D40" s="163" t="s">
+        <v>107</v>
+      </c>
+      <c r="E40" s="120" t="s">
         <v>115</v>
-      </c>
-      <c r="D40" s="135" t="s">
-        <v>108</v>
-      </c>
-      <c r="E40" s="120" t="s">
-        <v>116</v>
       </c>
       <c r="F40" s="85"/>
       <c r="G40" s="86" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H40" s="87"/>
       <c r="I40" s="87"/>
@@ -3366,16 +3375,16 @@
       <c r="AB40" s="87"/>
     </row>
     <row r="41" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A41" s="183"/>
-      <c r="B41" s="185"/>
-      <c r="C41" s="140"/>
-      <c r="D41" s="136"/>
+      <c r="A41" s="164"/>
+      <c r="B41" s="166"/>
+      <c r="C41" s="207"/>
+      <c r="D41" s="167"/>
       <c r="E41" s="121" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F41" s="85"/>
       <c r="G41" s="89" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H41" s="87"/>
       <c r="I41" s="87"/>
@@ -3400,18 +3409,18 @@
       <c r="AB41" s="87"/>
     </row>
     <row r="42" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A42" s="135">
+      <c r="A42" s="163">
         <v>20</v>
       </c>
-      <c r="B42" s="166" t="s">
+      <c r="B42" s="197" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" s="207"/>
+      <c r="D42" s="163" t="s">
+        <v>111</v>
+      </c>
+      <c r="E42" s="122" t="s">
         <v>119</v>
-      </c>
-      <c r="C42" s="140"/>
-      <c r="D42" s="135" t="s">
-        <v>112</v>
-      </c>
-      <c r="E42" s="122" t="s">
-        <v>120</v>
       </c>
       <c r="F42" s="85"/>
       <c r="G42" s="89"/>
@@ -3438,10 +3447,10 @@
       <c r="AB42" s="87"/>
     </row>
     <row r="43" spans="1:28" s="88" customFormat="1" ht="15" customHeight="1">
-      <c r="A43" s="136"/>
-      <c r="B43" s="167"/>
-      <c r="C43" s="141"/>
-      <c r="D43" s="136"/>
+      <c r="A43" s="167"/>
+      <c r="B43" s="198"/>
+      <c r="C43" s="208"/>
+      <c r="D43" s="167"/>
       <c r="E43" s="123"/>
       <c r="F43" s="90"/>
       <c r="G43" s="91"/>
@@ -3468,20 +3477,20 @@
       <c r="AB43" s="87"/>
     </row>
     <row r="44" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A44" s="133">
+      <c r="A44" s="199">
         <v>21</v>
       </c>
-      <c r="B44" s="137" t="s">
+      <c r="B44" s="204" t="s">
+        <v>120</v>
+      </c>
+      <c r="C44" s="209" t="s">
         <v>121</v>
       </c>
-      <c r="C44" s="142" t="s">
+      <c r="D44" s="199" t="s">
+        <v>107</v>
+      </c>
+      <c r="E44" s="124" t="s">
         <v>122</v>
-      </c>
-      <c r="D44" s="133" t="s">
-        <v>108</v>
-      </c>
-      <c r="E44" s="124" t="s">
-        <v>123</v>
       </c>
       <c r="F44" s="92"/>
       <c r="G44" s="93"/>
@@ -3508,14 +3517,14 @@
       <c r="AB44" s="94"/>
     </row>
     <row r="45" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A45" s="168"/>
-      <c r="B45" s="138"/>
-      <c r="C45" s="143"/>
-      <c r="D45" s="134"/>
+      <c r="A45" s="200"/>
+      <c r="B45" s="205"/>
+      <c r="C45" s="210"/>
+      <c r="D45" s="201"/>
       <c r="E45" s="125"/>
       <c r="F45" s="96"/>
       <c r="G45" s="97" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H45" s="94"/>
       <c r="I45" s="94"/>
@@ -3540,22 +3549,22 @@
       <c r="AB45" s="94"/>
     </row>
     <row r="46" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A46" s="133">
+      <c r="A46" s="199">
         <v>22</v>
       </c>
-      <c r="B46" s="131" t="s">
+      <c r="B46" s="202" t="s">
+        <v>124</v>
+      </c>
+      <c r="C46" s="210"/>
+      <c r="D46" s="199" t="s">
+        <v>111</v>
+      </c>
+      <c r="E46" s="126" t="s">
         <v>125</v>
-      </c>
-      <c r="C46" s="143"/>
-      <c r="D46" s="133" t="s">
-        <v>112</v>
-      </c>
-      <c r="E46" s="126" t="s">
-        <v>126</v>
       </c>
       <c r="F46" s="98"/>
       <c r="G46" s="92" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H46" s="94"/>
       <c r="I46" s="94"/>
@@ -3580,32 +3589,32 @@
       <c r="AB46" s="94"/>
     </row>
     <row r="47" spans="1:28" s="95" customFormat="1" ht="15" customHeight="1">
-      <c r="A47" s="134"/>
-      <c r="B47" s="132"/>
-      <c r="C47" s="144"/>
-      <c r="D47" s="134"/>
+      <c r="A47" s="201"/>
+      <c r="B47" s="203"/>
+      <c r="C47" s="211"/>
+      <c r="D47" s="201"/>
       <c r="E47" s="127"/>
       <c r="F47" s="99"/>
     </row>
     <row r="48" spans="1:28" ht="15" customHeight="1">
-      <c r="A48" s="145">
+      <c r="A48" s="135">
         <v>23</v>
       </c>
-      <c r="B48" s="164" t="s">
+      <c r="B48" s="195" t="s">
+        <v>127</v>
+      </c>
+      <c r="C48" s="189" t="s">
         <v>128</v>
       </c>
-      <c r="C48" s="158" t="s">
+      <c r="D48" s="143" t="s">
+        <v>107</v>
+      </c>
+      <c r="E48" s="128" t="s">
         <v>129</v>
-      </c>
-      <c r="D48" s="149" t="s">
-        <v>108</v>
-      </c>
-      <c r="E48" s="128" t="s">
-        <v>130</v>
       </c>
       <c r="F48" s="57"/>
       <c r="G48" s="75" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H48" s="30"/>
       <c r="I48" s="30"/>
@@ -3630,16 +3639,16 @@
       <c r="AB48" s="30"/>
     </row>
     <row r="49" spans="1:28" ht="15" customHeight="1">
-      <c r="A49" s="163"/>
-      <c r="B49" s="165"/>
-      <c r="C49" s="159"/>
-      <c r="D49" s="162"/>
+      <c r="A49" s="194"/>
+      <c r="B49" s="196"/>
+      <c r="C49" s="190"/>
+      <c r="D49" s="193"/>
       <c r="E49" s="129" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F49" s="69"/>
       <c r="G49" s="75" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H49" s="30"/>
       <c r="I49" s="30"/>
@@ -3664,25 +3673,25 @@
       <c r="AB49" s="30"/>
     </row>
     <row r="50" spans="1:28" ht="15" customHeight="1">
-      <c r="A50" s="145">
+      <c r="A50" s="135">
         <v>24</v>
       </c>
-      <c r="B50" s="147" t="s">
+      <c r="B50" s="181" t="s">
+        <v>133</v>
+      </c>
+      <c r="C50" s="190"/>
+      <c r="D50" s="143" t="s">
+        <v>111</v>
+      </c>
+      <c r="E50" s="130" t="s">
         <v>134</v>
-      </c>
-      <c r="C50" s="159"/>
-      <c r="D50" s="149" t="s">
-        <v>112</v>
-      </c>
-      <c r="E50" s="130" t="s">
-        <v>135</v>
       </c>
       <c r="F50" s="77"/>
       <c r="G50" s="72" t="s">
+        <v>135</v>
+      </c>
+      <c r="H50" s="75" t="s">
         <v>136</v>
-      </c>
-      <c r="H50" s="75" t="s">
-        <v>137</v>
       </c>
       <c r="I50" s="30"/>
       <c r="J50" s="30"/>
@@ -3706,16 +3715,16 @@
       <c r="AB50" s="30"/>
     </row>
     <row r="51" spans="1:28" ht="15" customHeight="1">
-      <c r="A51" s="146"/>
-      <c r="B51" s="148"/>
-      <c r="C51" s="160"/>
-      <c r="D51" s="150"/>
+      <c r="A51" s="180"/>
+      <c r="B51" s="182"/>
+      <c r="C51" s="191"/>
+      <c r="D51" s="183"/>
       <c r="E51" s="129" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F51" s="69"/>
       <c r="G51" s="69" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H51" s="30"/>
       <c r="I51" s="30"/>
@@ -3741,6 +3750,74 @@
     </row>
   </sheetData>
   <mergeCells count="84">
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C40:C43"/>
+    <mergeCell ref="C44:C47"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C36:C39"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C48:C51"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="A42:A43"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="C3:C10"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C11:C18"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C23:C26"/>
+    <mergeCell ref="C27:C34"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B33:B34"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="A13:A14"/>
@@ -3757,74 +3834,6 @@
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="C23:C26"/>
-    <mergeCell ref="C27:C34"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="C11:C18"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="C3:C10"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C36:C39"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C48:C51"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="A48:A49"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="A42:A43"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="A44:A45"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C40:C43"/>
-    <mergeCell ref="C44:C47"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -3942,14 +3951,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" customWidth="1"/>
-    <col min="2" max="2" width="85.28515625" customWidth="1"/>
-    <col min="3" max="3" width="47.7109375" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="2" max="2" width="85.33203125" customWidth="1"/>
+    <col min="3" max="3" width="47.6640625" customWidth="1"/>
     <col min="4" max="4" width="87" customWidth="1"/>
-    <col min="5" max="5" width="95.7109375" customWidth="1"/>
-    <col min="6" max="26" width="8.85546875" customWidth="1"/>
+    <col min="5" max="5" width="95.6640625" customWidth="1"/>
+    <col min="6" max="26" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -3980,7 +3989,7 @@
       <c r="Y1" s="4"/>
       <c r="Z1" s="4"/>
     </row>
-    <row r="2" spans="1:26" ht="15.95">
+    <row r="2" spans="1:26" ht="16">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -3988,10 +3997,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>141</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>5</v>
@@ -4018,7 +4027,7 @@
       <c r="Y2" s="8"/>
       <c r="Z2" s="8"/>
     </row>
-    <row r="3" spans="1:26" ht="15.95">
+    <row r="3" spans="1:26" ht="16">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -4026,10 +4035,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="33" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="34" t="s">
         <v>142</v>
-      </c>
-      <c r="D3" s="34" t="s">
-        <v>143</v>
       </c>
       <c r="E3" s="35" t="s">
         <v>10</v>
@@ -4057,21 +4066,21 @@
       <c r="Z3" s="10"/>
     </row>
     <row r="4" spans="1:26">
-      <c r="A4" s="218">
+      <c r="A4" s="212">
         <f>SUM(A3+1)</f>
         <v>2</v>
       </c>
-      <c r="B4" s="226" t="s">
+      <c r="B4" s="214" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="227" t="s">
+      <c r="C4" s="216" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="E4" s="218" t="s">
         <v>145</v>
-      </c>
-      <c r="E4" s="219" t="s">
-        <v>146</v>
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
@@ -4096,13 +4105,13 @@
       <c r="Z4" s="11"/>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A5" s="234"/>
-      <c r="B5" s="235"/>
-      <c r="C5" s="236"/>
+      <c r="A5" s="213"/>
+      <c r="B5" s="215"/>
+      <c r="C5" s="217"/>
       <c r="D5" s="36" t="s">
-        <v>147</v>
-      </c>
-      <c r="E5" s="234"/>
+        <v>146</v>
+      </c>
+      <c r="E5" s="213"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -4134,10 +4143,10 @@
         <v>72</v>
       </c>
       <c r="C6" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="34" t="s">
         <v>148</v>
-      </c>
-      <c r="D6" s="34" t="s">
-        <v>149</v>
       </c>
       <c r="E6" s="35" t="s">
         <v>73</v>
@@ -4173,27 +4182,27 @@
         <v>76</v>
       </c>
       <c r="C7" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="D7" s="34" t="s">
         <v>150</v>
-      </c>
-      <c r="D7" s="34" t="s">
-        <v>151</v>
       </c>
       <c r="E7" s="34" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:26">
-      <c r="A8" s="218">
+      <c r="A8" s="212">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B8" s="228" t="s">
+      <c r="B8" s="219" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="229" t="s">
-        <v>152</v>
-      </c>
-      <c r="D8" s="230" t="s">
+      <c r="C8" s="220" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8" s="221" t="s">
         <v>35</v>
       </c>
       <c r="E8" s="36" t="s">
@@ -4222,10 +4231,10 @@
       <c r="Z8" s="11"/>
     </row>
     <row r="9" spans="1:26">
-      <c r="A9" s="234"/>
-      <c r="B9" s="235"/>
-      <c r="C9" s="236"/>
-      <c r="D9" s="234"/>
+      <c r="A9" s="213"/>
+      <c r="B9" s="215"/>
+      <c r="C9" s="217"/>
+      <c r="D9" s="213"/>
       <c r="E9" s="36" t="s">
         <v>37</v>
       </c>
@@ -4252,17 +4261,17 @@
       <c r="Z9" s="11"/>
     </row>
     <row r="10" spans="1:26">
-      <c r="A10" s="210">
+      <c r="A10" s="224">
         <f>SUM(A8+1)</f>
         <v>6</v>
       </c>
-      <c r="B10" s="220" t="s">
+      <c r="B10" s="225" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="221" t="s">
-        <v>153</v>
-      </c>
-      <c r="D10" s="209" t="s">
+      <c r="C10" s="226" t="s">
+        <v>152</v>
+      </c>
+      <c r="D10" s="227" t="s">
         <v>40</v>
       </c>
       <c r="E10" s="34" t="s">
@@ -4291,10 +4300,10 @@
       <c r="Z10" s="13"/>
     </row>
     <row r="11" spans="1:26">
-      <c r="A11" s="234"/>
-      <c r="B11" s="235"/>
-      <c r="C11" s="236"/>
-      <c r="D11" s="234"/>
+      <c r="A11" s="213"/>
+      <c r="B11" s="215"/>
+      <c r="C11" s="217"/>
+      <c r="D11" s="213"/>
       <c r="E11" s="34" t="s">
         <v>41</v>
       </c>
@@ -4321,21 +4330,21 @@
       <c r="Z11" s="13"/>
     </row>
     <row r="12" spans="1:26">
-      <c r="A12" s="224">
+      <c r="A12" s="228">
         <f>SUM(A10+1)</f>
         <v>7</v>
       </c>
-      <c r="B12" s="225" t="s">
+      <c r="B12" s="229" t="s">
+        <v>153</v>
+      </c>
+      <c r="C12" s="222" t="s">
         <v>154</v>
       </c>
-      <c r="C12" s="222" t="s">
+      <c r="D12" s="223" t="s">
         <v>155</v>
       </c>
-      <c r="D12" s="223" t="s">
+      <c r="E12" s="14" t="s">
         <v>156</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>157</v>
       </c>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
@@ -4360,12 +4369,12 @@
       <c r="Z12" s="15"/>
     </row>
     <row r="13" spans="1:26">
-      <c r="A13" s="234"/>
-      <c r="B13" s="235"/>
-      <c r="C13" s="236"/>
-      <c r="D13" s="234"/>
+      <c r="A13" s="213"/>
+      <c r="B13" s="215"/>
+      <c r="C13" s="217"/>
+      <c r="D13" s="213"/>
       <c r="E13" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
@@ -4390,15 +4399,15 @@
       <c r="Z13" s="15"/>
     </row>
     <row r="14" spans="1:26">
-      <c r="A14" s="210">
+      <c r="A14" s="224">
         <f>SUM(A12+1)</f>
         <v>8</v>
       </c>
-      <c r="B14" s="220" t="s">
+      <c r="B14" s="225" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="221" t="s">
-        <v>159</v>
+      <c r="C14" s="226" t="s">
+        <v>158</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>46</v>
@@ -4408,14 +4417,14 @@
       </c>
     </row>
     <row r="15" spans="1:26">
-      <c r="A15" s="234"/>
-      <c r="B15" s="235"/>
-      <c r="C15" s="236"/>
+      <c r="A15" s="213"/>
+      <c r="B15" s="215"/>
+      <c r="C15" s="217"/>
       <c r="D15" s="34" t="s">
         <v>49</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:26">
@@ -4427,7 +4436,7 @@
         <v>56</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D16" s="36" t="s">
         <v>61</v>
@@ -4458,17 +4467,17 @@
       <c r="Z16" s="11"/>
     </row>
     <row r="17" spans="1:26">
-      <c r="A17" s="210">
+      <c r="A17" s="224">
         <f>A16+1</f>
         <v>10</v>
       </c>
       <c r="B17" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="215" t="s">
-        <v>162</v>
-      </c>
-      <c r="D17" s="209" t="s">
+      <c r="C17" s="230" t="s">
+        <v>161</v>
+      </c>
+      <c r="D17" s="227" t="s">
         <v>68</v>
       </c>
       <c r="E17" s="34" t="s">
@@ -4497,14 +4506,14 @@
       <c r="Z17" s="18"/>
     </row>
     <row r="18" spans="1:26">
-      <c r="A18" s="234"/>
+      <c r="A18" s="213"/>
       <c r="B18" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="236"/>
-      <c r="D18" s="234"/>
+      <c r="C18" s="217"/>
+      <c r="D18" s="213"/>
       <c r="E18" s="34" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F18" s="18"/>
       <c r="G18" s="18"/>
@@ -4528,7 +4537,7 @@
       <c r="Y18" s="18"/>
       <c r="Z18" s="18"/>
     </row>
-    <row r="19" spans="1:26" ht="15.95">
+    <row r="19" spans="1:26" ht="16">
       <c r="A19" s="16">
         <f>A17+1</f>
         <v>11</v>
@@ -4537,7 +4546,7 @@
         <v>92</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D19" s="41" t="s">
         <v>94</v>
@@ -4567,19 +4576,19 @@
       <c r="Y19" s="11"/>
       <c r="Z19" s="11"/>
     </row>
-    <row r="20" spans="1:26" ht="15.95">
+    <row r="20" spans="1:26" ht="16">
       <c r="A20" s="19">
         <f t="shared" ref="A20:A21" si="1">A19+1</f>
         <v>12</v>
       </c>
       <c r="B20" s="43" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="44" t="s">
         <v>165</v>
       </c>
-      <c r="C20" s="44" t="s">
+      <c r="D20" s="20" t="s">
         <v>166</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>167</v>
       </c>
       <c r="E20" s="21"/>
       <c r="F20" s="22"/>
@@ -4613,7 +4622,7 @@
         <v>15</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D21" s="46" t="s">
         <v>16</v>
@@ -4626,10 +4635,10 @@
         <v>14</v>
       </c>
       <c r="B22" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="C22" s="33" t="s">
         <v>169</v>
-      </c>
-      <c r="C22" s="33" t="s">
-        <v>170</v>
       </c>
       <c r="D22" s="34" t="s">
         <v>87</v>
@@ -4665,13 +4674,13 @@
         <v>15</v>
       </c>
       <c r="B23" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="C23" s="52" t="s">
         <v>171</v>
       </c>
-      <c r="C23" s="52" t="s">
+      <c r="D23" s="29" t="s">
         <v>172</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>173</v>
       </c>
       <c r="E23" s="53"/>
     </row>
@@ -4681,13 +4690,13 @@
         <v>16</v>
       </c>
       <c r="B24" s="47" t="s">
+        <v>173</v>
+      </c>
+      <c r="C24" s="54" t="s">
+        <v>167</v>
+      </c>
+      <c r="D24" s="55" t="s">
         <v>174</v>
-      </c>
-      <c r="C24" s="54" t="s">
-        <v>168</v>
-      </c>
-      <c r="D24" s="55" t="s">
-        <v>175</v>
       </c>
       <c r="E24" s="56"/>
       <c r="F24" s="11"/>
@@ -4713,18 +4722,18 @@
       <c r="Z24" s="11"/>
     </row>
     <row r="25" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A25" s="210">
+      <c r="A25" s="224">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="B25" s="214" t="s">
-        <v>106</v>
-      </c>
-      <c r="C25" s="215" t="s">
-        <v>176</v>
-      </c>
-      <c r="D25" s="211" t="s">
-        <v>109</v>
+      <c r="B25" s="234" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="230" t="s">
+        <v>175</v>
+      </c>
+      <c r="D25" s="231" t="s">
+        <v>108</v>
       </c>
       <c r="E25" s="35" t="s">
         <v>91</v>
@@ -4752,12 +4761,12 @@
       <c r="Z25" s="24"/>
     </row>
     <row r="26" spans="1:26" ht="15" customHeight="1">
-      <c r="A26" s="234"/>
-      <c r="B26" s="235"/>
-      <c r="C26" s="236"/>
-      <c r="D26" s="234"/>
+      <c r="A26" s="213"/>
+      <c r="B26" s="215"/>
+      <c r="C26" s="217"/>
+      <c r="D26" s="213"/>
       <c r="E26" s="34" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F26" s="24"/>
       <c r="G26" s="24"/>
@@ -4787,13 +4796,13 @@
         <v>18</v>
       </c>
       <c r="B27" s="48" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E27" s="26"/>
       <c r="F27" s="11"/>
@@ -4819,21 +4828,21 @@
       <c r="Z27" s="11"/>
     </row>
     <row r="28" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A28" s="216">
+      <c r="A28" s="235">
         <f>A27+1</f>
         <v>19</v>
       </c>
-      <c r="B28" s="217" t="s">
-        <v>132</v>
-      </c>
-      <c r="C28" s="215" t="s">
-        <v>178</v>
-      </c>
-      <c r="D28" s="209" t="s">
+      <c r="B28" s="236" t="s">
+        <v>131</v>
+      </c>
+      <c r="C28" s="230" t="s">
+        <v>177</v>
+      </c>
+      <c r="D28" s="227" t="s">
+        <v>129</v>
+      </c>
+      <c r="E28" s="34" t="s">
         <v>130</v>
-      </c>
-      <c r="E28" s="34" t="s">
-        <v>131</v>
       </c>
       <c r="F28" s="10"/>
       <c r="G28" s="10"/>
@@ -4858,12 +4867,12 @@
       <c r="Z28" s="10"/>
     </row>
     <row r="29" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A29" s="234"/>
-      <c r="B29" s="235"/>
-      <c r="C29" s="236"/>
-      <c r="D29" s="234"/>
+      <c r="A29" s="213"/>
+      <c r="B29" s="215"/>
+      <c r="C29" s="217"/>
+      <c r="D29" s="213"/>
       <c r="E29" s="34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
@@ -4888,21 +4897,21 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A30" s="218">
+      <c r="A30" s="212">
         <f>A28+1</f>
         <v>20</v>
       </c>
-      <c r="B30" s="212" t="s">
-        <v>135</v>
-      </c>
-      <c r="C30" s="213" t="s">
+      <c r="B30" s="232" t="s">
+        <v>134</v>
+      </c>
+      <c r="C30" s="233" t="s">
+        <v>178</v>
+      </c>
+      <c r="D30" s="218" t="s">
         <v>179</v>
       </c>
-      <c r="D30" s="219" t="s">
-        <v>180</v>
-      </c>
       <c r="E30" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F30" s="11"/>
       <c r="G30" s="11"/>
@@ -4927,12 +4936,12 @@
       <c r="Z30" s="11"/>
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A31" s="234"/>
-      <c r="B31" s="235"/>
-      <c r="C31" s="236"/>
-      <c r="D31" s="234"/>
+      <c r="A31" s="213"/>
+      <c r="B31" s="215"/>
+      <c r="C31" s="217"/>
+      <c r="D31" s="213"/>
       <c r="E31" s="41" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F31" s="11"/>
       <c r="G31" s="11"/>
@@ -4962,13 +4971,13 @@
         <v>21</v>
       </c>
       <c r="B32" s="45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D32" s="35" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E32" s="27"/>
     </row>
@@ -4978,13 +4987,13 @@
         <v>22</v>
       </c>
       <c r="B33" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="D33" s="34" t="s">
         <v>119</v>
-      </c>
-      <c r="C33" s="33" t="s">
-        <v>182</v>
-      </c>
-      <c r="D33" s="34" t="s">
-        <v>120</v>
       </c>
       <c r="E33" s="27"/>
       <c r="F33" s="24"/>
@@ -5015,14 +5024,14 @@
         <v>24</v>
       </c>
       <c r="B34" s="41" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D34" s="41"/>
       <c r="E34" s="36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F34" s="11"/>
       <c r="G34" s="11"/>
@@ -11810,27 +11819,6 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="C17:C18"/>
     <mergeCell ref="D17:D18"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="D25:D26"/>
@@ -11844,6 +11832,27 @@
     <mergeCell ref="D28:D29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="D30:D31"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
@@ -11934,17 +11943,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f0b0792d-d654-4f32-9135-0cf693c22f67">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c805177d-b823-4c7f-87f1-c3fe271a3d2d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD90A491793F574D833EEF3FF0869CA1" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b15b8ac1b6df1795c032a72689c8e15f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f0b0792d-d654-4f32-9135-0cf693c22f67" xmlns:ns3="c805177d-b823-4c7f-87f1-c3fe271a3d2d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7e45a94f909e329f9a8ac4529b6db8ce" ns2:_="" ns3:_="">
     <xsd:import namespace="f0b0792d-d654-4f32-9135-0cf693c22f67"/>
@@ -12199,16 +12197,53 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f0b0792d-d654-4f32-9135-0cf693c22f67">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c805177d-b823-4c7f-87f1-c3fe271a3d2d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1393095-9EBA-4193-AB4B-17269DE767FD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1393095-9EBA-4193-AB4B-17269DE767FD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E1BC49D-499B-4FD5-B4A6-90CBD04CEF93}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{451CC68B-C786-4554-BF8A-BED96CCD5B5C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f0b0792d-d654-4f32-9135-0cf693c22f67"/>
+    <ds:schemaRef ds:uri="c805177d-b823-4c7f-87f1-c3fe271a3d2d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{451CC68B-C786-4554-BF8A-BED96CCD5B5C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E1BC49D-499B-4FD5-B4A6-90CBD04CEF93}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f0b0792d-d654-4f32-9135-0cf693c22f67"/>
+    <ds:schemaRef ds:uri="c805177d-b823-4c7f-87f1-c3fe271a3d2d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>